<commit_message>
Research: manuscript builder, verified references, formatted thesis and preview
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0186tGPQJ67bKVgWZR7S3c4o
</commit_message>
<xml_diff>
--- a/research/output/tables/all_results.xlsx
+++ b/research/output/tables/all_results.xlsx
@@ -172,7 +172,7 @@
     <t>Effect on doctor relationship</t>
   </si>
   <si>
-    <t>AI chatbots</t>
+    <t>AI chatbots*</t>
   </si>
   <si>
     <t>Search engines</t>
@@ -19640,10 +19640,10 @@
         <v>41</v>
       </c>
       <c r="D2">
-        <v>234</v>
+        <v>266</v>
       </c>
       <c r="E2">
-        <v>78</v>
+        <v>88.7</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -26605,41 +26605,41 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
+        <v>206</v>
+      </c>
+      <c r="C2" t="s">
         <v>205</v>
       </c>
-      <c r="C2" t="s">
-        <v>204</v>
-      </c>
       <c r="D2">
-        <v>0.419</v>
+        <v>0.607</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C3" t="s">
         <v>205</v>
       </c>
       <c r="D3">
-        <v>0.607</v>
+        <v>0.419</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" t="s">
         <v>206</v>
-      </c>
-      <c r="C4" t="s">
-        <v>204</v>
       </c>
       <c r="D4">
         <v>0.669</v>

</xml_diff>

<commit_message>
Research: address external review - mediation b paths, elevated-HA label, hedged claims, refs
- Mediation: report b path adjusted for the predictor (indirect = a x b = c - c')
- SHAI >= 18 relabelled 'elevated' (not 'clinically relevant'); prevalence at 29 added
- Tool count uses the study's AI-user definition; Holm pairwise p reported
- Post-hoc power removed; abstract shortened and hedged; objectives cut to four
- Behavioural findings marked exploratory; H3/H4 verdicts stated
- Limitations: unused Arabic versions and response-option order
- ClinicalTrials.gov description corrected; missing DOIs and entry details added

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0186tGPQJ67bKVgWZR7S3c4o
</commit_message>
<xml_diff>
--- a/research/output/tables/all_results.xlsx
+++ b/research/output/tables/all_results.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3292" uniqueCount="674">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3300" uniqueCount="675">
   <si>
     <t>Variable</t>
   </si>
@@ -1833,6 +1833,9 @@
   </si>
   <si>
     <t>Indirect</t>
+  </si>
+  <si>
+    <t>b (M -&gt; Y | X)</t>
   </si>
   <si>
     <t>CSS_distress ~ X</t>
@@ -2894,7 +2897,7 @@
         <v>0.048</v>
       </c>
       <c r="I2">
-        <v>0.23</v>
+        <v>0.221</v>
       </c>
       <c r="J2">
         <v>0.166</v>
@@ -2929,7 +2932,7 @@
         <v>0.11</v>
       </c>
       <c r="I3">
-        <v>0.192</v>
+        <v>0.235</v>
       </c>
       <c r="J3">
         <v>0.132</v>
@@ -2999,7 +3002,7 @@
         <v>0.038</v>
       </c>
       <c r="I5">
-        <v>0.132</v>
+        <v>0.192</v>
       </c>
       <c r="J5">
         <v>0.035</v>
@@ -3034,7 +3037,7 @@
         <v>0.096</v>
       </c>
       <c r="I6">
-        <v>0.144</v>
+        <v>0.175</v>
       </c>
       <c r="J6">
         <v>0.063</v>
@@ -3069,7 +3072,7 @@
         <v>0.025</v>
       </c>
       <c r="I7">
-        <v>0.115</v>
+        <v>0.132</v>
       </c>
       <c r="J7">
         <v>0.029</v>
@@ -3104,7 +3107,7 @@
         <v>1</v>
       </c>
       <c r="I8">
-        <v>0.094</v>
+        <v>0.062</v>
       </c>
       <c r="J8">
         <v>0.177</v>
@@ -3118,34 +3121,34 @@
         <v>218</v>
       </c>
       <c r="B9">
-        <v>0.23</v>
+        <v>0.221</v>
       </c>
       <c r="C9">
-        <v>0.192</v>
+        <v>0.235</v>
       </c>
       <c r="D9">
         <v>0.221</v>
       </c>
       <c r="E9">
+        <v>0.192</v>
+      </c>
+      <c r="F9">
+        <v>0.175</v>
+      </c>
+      <c r="G9">
         <v>0.132</v>
       </c>
-      <c r="F9">
-        <v>0.144</v>
-      </c>
-      <c r="G9">
-        <v>0.115</v>
-      </c>
       <c r="H9">
-        <v>0.094</v>
+        <v>0.062</v>
       </c>
       <c r="I9">
         <v>1</v>
       </c>
       <c r="J9">
-        <v>0.322</v>
+        <v>0.233</v>
       </c>
       <c r="K9">
-        <v>-0.08500000000000001</v>
+        <v>-0.063</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -3174,7 +3177,7 @@
         <v>0.177</v>
       </c>
       <c r="I10">
-        <v>0.322</v>
+        <v>0.233</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -3209,7 +3212,7 @@
         <v>0.053</v>
       </c>
       <c r="I11">
-        <v>-0.08500000000000001</v>
+        <v>-0.063</v>
       </c>
       <c r="J11">
         <v>-0.08500000000000001</v>
@@ -3286,13 +3289,13 @@
         <v>0.4604</v>
       </c>
       <c r="I2">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
       <c r="J2">
-        <v>0.0074</v>
+        <v>0.0068</v>
       </c>
       <c r="K2">
-        <v>0.002</v>
+        <v>0.0019</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -3321,13 +3324,13 @@
         <v>0.08690000000000001</v>
       </c>
       <c r="I3">
-        <v>0.0019</v>
+        <v>0.0001</v>
       </c>
       <c r="J3">
-        <v>0.0373</v>
+        <v>0.0364</v>
       </c>
       <c r="K3">
-        <v>0.2625</v>
+        <v>0.2784</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -3353,7 +3356,7 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>0.0022</v>
+        <v>0.0021</v>
       </c>
       <c r="I4">
         <v>0.0003</v>
@@ -3391,13 +3394,13 @@
         <v>0.543</v>
       </c>
       <c r="I5">
-        <v>0.0373</v>
+        <v>0.0018</v>
       </c>
       <c r="J5">
         <v>0.5718</v>
       </c>
       <c r="K5">
-        <v>0.1909</v>
+        <v>0.2024</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -3426,10 +3429,10 @@
         <v>0.1469</v>
       </c>
       <c r="I6">
-        <v>0.0223</v>
+        <v>0.0043</v>
       </c>
       <c r="J6">
-        <v>0.3433</v>
+        <v>0.3531</v>
       </c>
       <c r="K6">
         <v>0.543</v>
@@ -3461,7 +3464,7 @@
         <v>0.6685</v>
       </c>
       <c r="I7">
-        <v>0.075</v>
+        <v>0.0364</v>
       </c>
       <c r="J7">
         <v>0.6368</v>
@@ -3481,7 +3484,7 @@
         <v>0.08690000000000001</v>
       </c>
       <c r="D8">
-        <v>0.0022</v>
+        <v>0.0021</v>
       </c>
       <c r="E8">
         <v>0.543</v>
@@ -3496,10 +3499,10 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>0.1513</v>
+        <v>0.3555</v>
       </c>
       <c r="J8">
-        <v>0.004</v>
+        <v>0.0038</v>
       </c>
       <c r="K8">
         <v>0.4262</v>
@@ -3510,34 +3513,34 @@
         <v>218</v>
       </c>
       <c r="B9">
+        <v>0.0003</v>
+      </c>
+      <c r="C9">
         <v>0.0001</v>
-      </c>
-      <c r="C9">
-        <v>0.0019</v>
       </c>
       <c r="D9">
         <v>0.0003</v>
       </c>
       <c r="E9">
-        <v>0.0373</v>
+        <v>0.0018</v>
       </c>
       <c r="F9">
-        <v>0.0223</v>
+        <v>0.0043</v>
       </c>
       <c r="G9">
-        <v>0.075</v>
+        <v>0.0364</v>
       </c>
       <c r="H9">
-        <v>0.1513</v>
+        <v>0.3555</v>
       </c>
       <c r="I9">
         <v>0</v>
       </c>
       <c r="J9">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="K9">
-        <v>0.1909</v>
+        <v>0.3531</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -3545,10 +3548,10 @@
         <v>219</v>
       </c>
       <c r="B10">
-        <v>0.0074</v>
+        <v>0.0068</v>
       </c>
       <c r="C10">
-        <v>0.0373</v>
+        <v>0.0364</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -3557,22 +3560,22 @@
         <v>0.5718</v>
       </c>
       <c r="F10">
-        <v>0.3433</v>
+        <v>0.3531</v>
       </c>
       <c r="G10">
         <v>0.6368</v>
       </c>
       <c r="H10">
-        <v>0.004</v>
+        <v>0.0038</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>0.1909</v>
+        <v>0.2024</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -3580,16 +3583,16 @@
         <v>220</v>
       </c>
       <c r="B11">
-        <v>0.002</v>
+        <v>0.0019</v>
       </c>
       <c r="C11">
-        <v>0.2625</v>
+        <v>0.2784</v>
       </c>
       <c r="D11">
         <v>0.4435</v>
       </c>
       <c r="E11">
-        <v>0.1909</v>
+        <v>0.2024</v>
       </c>
       <c r="F11">
         <v>0.543</v>
@@ -3601,10 +3604,10 @@
         <v>0.4262</v>
       </c>
       <c r="I11">
-        <v>0.1909</v>
+        <v>0.3531</v>
       </c>
       <c r="J11">
-        <v>0.1909</v>
+        <v>0.2024</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -22879,7 +22882,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -23022,19 +23025,19 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C7" t="s">
-        <v>590</v>
+        <v>595</v>
       </c>
       <c r="D7">
-        <v>0.4621</v>
+        <v>0.3521</v>
       </c>
       <c r="E7">
-        <v>0.361</v>
+        <v>0.2284</v>
       </c>
       <c r="F7">
-        <v>0.5632</v>
+        <v>0.4758</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -23048,16 +23051,16 @@
         <v>587</v>
       </c>
       <c r="C8" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="D8">
-        <v>0.3432</v>
+        <v>0.4621</v>
       </c>
       <c r="E8">
-        <v>0.2309</v>
+        <v>0.361</v>
       </c>
       <c r="F8">
-        <v>0.4555</v>
+        <v>0.5632</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -23071,16 +23074,16 @@
         <v>587</v>
       </c>
       <c r="C9" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="D9">
-        <v>0.2796</v>
+        <v>0.3432</v>
       </c>
       <c r="E9">
-        <v>0.1659</v>
+        <v>0.2309</v>
       </c>
       <c r="F9">
-        <v>0.3933</v>
+        <v>0.4555</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -23094,19 +23097,19 @@
         <v>587</v>
       </c>
       <c r="C10" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D10">
-        <v>0.1545</v>
+        <v>0.2796</v>
       </c>
       <c r="E10">
-        <v>0.0296</v>
+        <v>0.1659</v>
       </c>
       <c r="F10">
-        <v>0.2794</v>
+        <v>0.3933</v>
       </c>
       <c r="G10">
-        <v>0.0155</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -23117,19 +23120,19 @@
         <v>587</v>
       </c>
       <c r="C11" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="D11">
-        <v>0.1251</v>
+        <v>0.1545</v>
       </c>
       <c r="E11">
-        <v>0.06619999999999999</v>
+        <v>0.0296</v>
       </c>
       <c r="F11">
-        <v>0.1994</v>
+        <v>0.2794</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>0.0155</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -23137,19 +23140,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C12" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="D12">
-        <v>0.4618</v>
+        <v>0.1251</v>
       </c>
       <c r="E12">
-        <v>0.3585</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="F12">
-        <v>0.5652</v>
+        <v>0.1994</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -23160,22 +23163,22 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C13" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D13">
-        <v>0.4782</v>
+        <v>0.2706</v>
       </c>
       <c r="E13">
-        <v>0.3762</v>
+        <v>0.1396</v>
       </c>
       <c r="F13">
-        <v>0.5802</v>
+        <v>0.4016</v>
       </c>
       <c r="G13">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -23186,19 +23189,19 @@
         <v>588</v>
       </c>
       <c r="C14" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="D14">
-        <v>0.2249</v>
+        <v>0.4618</v>
       </c>
       <c r="E14">
-        <v>0.1108</v>
+        <v>0.3585</v>
       </c>
       <c r="F14">
-        <v>0.3389</v>
+        <v>0.5652</v>
       </c>
       <c r="G14">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -23209,19 +23212,19 @@
         <v>588</v>
       </c>
       <c r="C15" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="D15">
-        <v>0.0051</v>
+        <v>0.4782</v>
       </c>
       <c r="E15">
-        <v>-0.1109</v>
+        <v>0.3762</v>
       </c>
       <c r="F15">
-        <v>0.121</v>
+        <v>0.5802</v>
       </c>
       <c r="G15">
-        <v>0.9316</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -23232,19 +23235,19 @@
         <v>588</v>
       </c>
       <c r="C16" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D16">
-        <v>0.2198</v>
+        <v>0.2249</v>
       </c>
       <c r="E16">
-        <v>0.1579</v>
+        <v>0.1108</v>
       </c>
       <c r="F16">
-        <v>0.2928</v>
+        <v>0.3389</v>
       </c>
       <c r="G16">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -23252,22 +23255,22 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C17" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D17">
-        <v>0.4925</v>
+        <v>0.0051</v>
       </c>
       <c r="E17">
-        <v>0.39</v>
+        <v>-0.1109</v>
       </c>
       <c r="F17">
-        <v>0.595</v>
+        <v>0.121</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>0.9316</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -23275,19 +23278,19 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C18" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D18">
-        <v>0.4532</v>
+        <v>0.2198</v>
       </c>
       <c r="E18">
-        <v>0.3517</v>
+        <v>0.1579</v>
       </c>
       <c r="F18">
-        <v>0.5546</v>
+        <v>0.2928</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -23298,19 +23301,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C19" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="D19">
-        <v>0.4694</v>
+        <v>0.4759</v>
       </c>
       <c r="E19">
-        <v>0.3666</v>
+        <v>0.345</v>
       </c>
       <c r="F19">
-        <v>0.5721000000000001</v>
+        <v>0.6068</v>
       </c>
       <c r="G19">
         <v>0</v>
@@ -23324,16 +23327,16 @@
         <v>589</v>
       </c>
       <c r="C20" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="D20">
-        <v>0.3215</v>
+        <v>0.4925</v>
       </c>
       <c r="E20">
-        <v>0.2093</v>
+        <v>0.39</v>
       </c>
       <c r="F20">
-        <v>0.4337</v>
+        <v>0.595</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -23347,18 +23350,110 @@
         <v>589</v>
       </c>
       <c r="C21" t="s">
+        <v>597</v>
+      </c>
+      <c r="D21">
+        <v>0.4532</v>
+      </c>
+      <c r="E21">
+        <v>0.3517</v>
+      </c>
+      <c r="F21">
+        <v>0.5546</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>589</v>
+      </c>
+      <c r="C22" t="s">
+        <v>592</v>
+      </c>
+      <c r="D22">
+        <v>0.4694</v>
+      </c>
+      <c r="E22">
+        <v>0.3666</v>
+      </c>
+      <c r="F22">
+        <v>0.5721000000000001</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>589</v>
+      </c>
+      <c r="C23" t="s">
+        <v>593</v>
+      </c>
+      <c r="D23">
+        <v>0.3215</v>
+      </c>
+      <c r="E23">
+        <v>0.2093</v>
+      </c>
+      <c r="F23">
+        <v>0.4337</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>589</v>
+      </c>
+      <c r="C24" t="s">
         <v>594</v>
       </c>
-      <c r="D21">
+      <c r="D24">
         <v>0.1478</v>
       </c>
-      <c r="E21">
+      <c r="E24">
         <v>0.0857</v>
       </c>
-      <c r="F21">
+      <c r="F24">
         <v>0.2186</v>
       </c>
-      <c r="G21">
+      <c r="G24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>589</v>
+      </c>
+      <c r="C25" t="s">
+        <v>595</v>
+      </c>
+      <c r="D25">
+        <v>0.3002</v>
+      </c>
+      <c r="E25">
+        <v>0.1796</v>
+      </c>
+      <c r="F25">
+        <v>0.4207</v>
+      </c>
+      <c r="G25">
         <v>0</v>
       </c>
     </row>
@@ -23391,7 +23486,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="C2">
         <v>0.0737</v>
@@ -23408,7 +23503,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="C3">
         <v>0.1263</v>
@@ -23425,7 +23520,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C4">
         <v>0.0687</v>
@@ -23442,7 +23537,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="C5">
         <v>-0.0438</v>
@@ -23466,10 +23561,10 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="B1" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="C1" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D1" t="s">
         <v>561</v>
@@ -23489,13 +23584,13 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="C2">
         <v>0.1007</v>
       </c>
       <c r="D2" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="E2">
         <v>0.3431</v>
@@ -23512,13 +23607,13 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="C3">
         <v>-0.1404</v>
       </c>
       <c r="D3" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E3">
         <v>0.4687</v>
@@ -23541,7 +23636,7 @@
         <v>0.0636</v>
       </c>
       <c r="D4" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E4">
         <v>0.6631</v>
@@ -23558,13 +23653,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="C5">
         <v>0.0042</v>
       </c>
       <c r="D5" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E5">
         <v>0.9769</v>
@@ -23587,7 +23682,7 @@
         <v>-0.0634</v>
       </c>
       <c r="D6" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E6">
         <v>0.754</v>
@@ -23604,13 +23699,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="C7">
         <v>-0.1769</v>
       </c>
       <c r="D7" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E7">
         <v>0.292</v>
@@ -23627,13 +23722,13 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="C8">
         <v>-0.1394</v>
       </c>
       <c r="D8" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="E8">
         <v>0.0684</v>
@@ -23968,10 +24063,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="B1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="C1" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D1" t="s">
         <v>543</v>
@@ -23988,7 +24083,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="C2">
         <v>0.6153</v>
@@ -24008,7 +24103,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="C3">
         <v>0.6905</v>
@@ -24028,7 +24123,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="C4">
         <v>0.7655999999999999</v>
@@ -24064,13 +24159,13 @@
         <v>32</v>
       </c>
       <c r="E1" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F1" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G1" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -24081,10 +24176,10 @@
         <v>254</v>
       </c>
       <c r="C2" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D2" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E2">
         <v>0.8571</v>
@@ -24104,10 +24199,10 @@
         <v>255</v>
       </c>
       <c r="C3" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D3" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E3">
         <v>0.6538</v>
@@ -24131,13 +24226,13 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="B1" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="C1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="D1" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="E1" t="s">
         <v>214</v>
@@ -24151,10 +24246,10 @@
         <v>254</v>
       </c>
       <c r="C2" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D2" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E2">
         <v>0.0043</v>
@@ -24168,10 +24263,10 @@
         <v>255</v>
       </c>
       <c r="C3" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D3" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E3">
         <v>0.9893</v>
@@ -24182,13 +24277,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="C4" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D4" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E4">
         <v>0.6168</v>
@@ -24199,13 +24294,13 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="C5" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D5" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="E5">
         <v>0.9154</v>
@@ -24216,13 +24311,13 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="C6" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D6" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E6">
         <v>0.5339</v>
@@ -24233,13 +24328,13 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="C7" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="D7" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="E7">
         <v>0.6138</v>
@@ -24253,10 +24348,10 @@
         <v>558</v>
       </c>
       <c r="C8" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D8" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E8">
         <v>0.2515</v>
@@ -24274,16 +24369,16 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="B1" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="C1" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="F1" t="s">
         <v>561</v>
@@ -24309,7 +24404,7 @@
         <v>0.4983</v>
       </c>
       <c r="F2" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -24332,7 +24427,7 @@
         <v>0.4502</v>
       </c>
       <c r="F3" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -24355,7 +24450,7 @@
         <v>0.5725</v>
       </c>
       <c r="F4" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -24378,7 +24473,7 @@
         <v>0.3512</v>
       </c>
       <c r="F5" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="G5">
         <v>0.0209</v>
@@ -24401,7 +24496,7 @@
         <v>0.4656</v>
       </c>
       <c r="F6" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="G6">
         <v>0.0011</v>
@@ -24424,7 +24519,7 @@
         <v>0.4851</v>
       </c>
       <c r="F7" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -24447,7 +24542,7 @@
         <v>0.2335</v>
       </c>
       <c r="F8" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="G8">
         <v>0.4022</v>
@@ -24470,7 +24565,7 @@
         <v>0.5508999999999999</v>
       </c>
       <c r="F9" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -24493,7 +24588,7 @@
         <v>0.5004</v>
       </c>
       <c r="F10" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="G10">
         <v>0.0001</v>
@@ -24516,7 +24611,7 @@
         <v>0.3586</v>
       </c>
       <c r="F11" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="G11">
         <v>0.0317</v>
@@ -24539,7 +24634,7 @@
         <v>0.3389</v>
       </c>
       <c r="F12" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="G12">
         <v>0.1329</v>
@@ -24550,7 +24645,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C13" t="s">
         <v>30</v>
@@ -24562,7 +24657,7 @@
         <v>0.4617</v>
       </c>
       <c r="F13" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -24573,7 +24668,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -24585,7 +24680,7 @@
         <v>0.4801</v>
       </c>
       <c r="F14" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G14">
         <v>0.0001</v>
@@ -24608,7 +24703,7 @@
         <v>0.3938</v>
       </c>
       <c r="F15" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -24631,7 +24726,7 @@
         <v>0.4736</v>
       </c>
       <c r="F16" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -24654,7 +24749,7 @@
         <v>0.6066</v>
       </c>
       <c r="F17" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="G17">
         <v>0.0001</v>
@@ -24677,7 +24772,7 @@
         <v>0.5031</v>
       </c>
       <c r="F18" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -24700,7 +24795,7 @@
         <v>0.3976</v>
       </c>
       <c r="F19" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="G19">
         <v>0.0001</v>
@@ -24724,7 +24819,7 @@
         <v>117</v>
       </c>
       <c r="D1" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E1" t="s">
         <v>74</v>
@@ -25184,16 +25279,16 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="B1" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="C1" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="D1" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="E1" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="F1" t="s">
         <v>222</v>
@@ -25205,7 +25300,7 @@
         <v>223</v>
       </c>
       <c r="I1" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
     </row>
     <row r="2" spans="1:9">

</xml_diff>